<commit_message>
end to end analysis
</commit_message>
<xml_diff>
--- a/baseline_hepaus_pars.xlsx
+++ b/baseline_hepaus_pars.xlsx
@@ -540,76 +540,76 @@
         <v>25</v>
       </c>
       <c r="B2">
-        <v>17.35018532827379</v>
+        <v>18.48417578649617</v>
       </c>
       <c r="C2">
-        <v>308.1625472254378</v>
+        <v>336.6093924101857</v>
       </c>
       <c r="D2">
-        <v>379.702063421468</v>
+        <v>362.6634693098511</v>
       </c>
       <c r="E2">
-        <v>17.81217735045846</v>
+        <v>19.51076314459439</v>
       </c>
       <c r="F2">
-        <v>293.9405821174268</v>
+        <v>334.373192306528</v>
       </c>
       <c r="G2">
-        <v>384.4022276754265</v>
+        <v>375.4590379768111</v>
       </c>
       <c r="H2">
-        <v>21.24526949598164</v>
+        <v>21.86579141979038</v>
       </c>
       <c r="I2">
-        <v>90.42180651768149</v>
+        <v>101.9467323267382</v>
       </c>
       <c r="J2">
-        <v>688.1715947024986</v>
+        <v>709.3782833634586</v>
       </c>
       <c r="K2">
-        <v>21.40691555068578</v>
+        <v>24.87729082341614</v>
       </c>
       <c r="L2">
-        <v>89.4655047679428</v>
+        <v>104.2095467127555</v>
       </c>
       <c r="M2">
-        <v>689.6491914107214</v>
+        <v>739.1165571425611</v>
       </c>
       <c r="N2">
-        <v>1.20543568206766</v>
+        <v>1.246137635074309</v>
       </c>
       <c r="O2">
-        <v>2.142456006707206</v>
+        <v>2.391584698141559</v>
       </c>
       <c r="P2">
-        <v>9.096141078721722</v>
+        <v>6.982498587646266</v>
       </c>
       <c r="Q2">
-        <v>1.20543568206766</v>
+        <v>1.246137635074309</v>
       </c>
       <c r="R2">
-        <v>1.99862551720854</v>
+        <v>2.246608773545434</v>
       </c>
       <c r="S2">
-        <v>8.992539040527834</v>
+        <v>7.008045735217956</v>
       </c>
       <c r="T2">
-        <v>0.6151393162958267</v>
+        <v>0.6170378583123783</v>
       </c>
       <c r="U2">
-        <v>0.6786997806346581</v>
+        <v>0.6881388067942998</v>
       </c>
       <c r="V2">
-        <v>0.9562125838918474</v>
+        <v>1.068426268265968</v>
       </c>
       <c r="W2">
-        <v>0.6151393162958267</v>
+        <v>0.6167506274594454</v>
       </c>
       <c r="X2">
-        <v>0.6124018349142032</v>
+        <v>0.6210989077072122</v>
       </c>
       <c r="Y2">
-        <v>0.9374721360948978</v>
+        <v>1.02951459833655</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -617,76 +617,76 @@
         <v>26</v>
       </c>
       <c r="B3">
-        <v>0.05491685137255099</v>
+        <v>0.0529089448780045</v>
       </c>
       <c r="C3">
-        <v>0.01978299735190353</v>
+        <v>0.01972089867094264</v>
       </c>
       <c r="D3">
-        <v>0.01891828336329808</v>
+        <v>0.01915586180581189</v>
       </c>
       <c r="E3">
-        <v>0.05369126234472001</v>
+        <v>0.05109198959676253</v>
       </c>
       <c r="F3">
-        <v>0.02056094604294263</v>
+        <v>0.02032383817648103</v>
       </c>
       <c r="G3">
-        <v>0.01892821395888496</v>
+        <v>0.0191811790910337</v>
       </c>
       <c r="H3">
-        <v>0.05429699378345434</v>
+        <v>0.05337702947432052</v>
       </c>
       <c r="I3">
-        <v>0.0224663946525725</v>
+        <v>0.02204566892543731</v>
       </c>
       <c r="J3">
-        <v>0.01889594420981888</v>
+        <v>0.01888665172255115</v>
       </c>
       <c r="K3">
-        <v>0.05369665224983282</v>
+        <v>0.04913473409093153</v>
       </c>
       <c r="L3">
-        <v>0.02268632464744934</v>
+        <v>0.02215946038287137</v>
       </c>
       <c r="M3">
-        <v>0.01889548993635298</v>
+        <v>0.01887216237367744</v>
       </c>
       <c r="N3">
-        <v>0.101889274834068</v>
+        <v>0.09804766534194742</v>
       </c>
       <c r="O3">
-        <v>0.04944613164409468</v>
+        <v>0.04558949978006736</v>
       </c>
       <c r="P3">
-        <v>0.02428746796940192</v>
+        <v>0.02626313639551821</v>
       </c>
       <c r="Q3">
-        <v>0.101889274834068</v>
+        <v>0.09804766534194742</v>
       </c>
       <c r="R3">
-        <v>0.05045569840354656</v>
+        <v>0.04640989286416679</v>
       </c>
       <c r="S3">
-        <v>0.024352482228769</v>
+        <v>0.02621573227731289</v>
       </c>
       <c r="T3">
-        <v>0.1138601273686702</v>
+        <v>0.1099217914334042</v>
       </c>
       <c r="U3">
-        <v>0.05895904124852858</v>
+        <v>0.05494639158149636</v>
       </c>
       <c r="V3">
-        <v>0.02891227687330087</v>
+        <v>0.02678790885682546</v>
       </c>
       <c r="W3">
-        <v>0.1138601273686702</v>
+        <v>0.1105047786779234</v>
       </c>
       <c r="X3">
-        <v>0.06047695208639974</v>
+        <v>0.05626047406919778</v>
       </c>
       <c r="Y3">
-        <v>0.02895081790571305</v>
+        <v>0.02706801197766756</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -694,76 +694,76 @@
         <v>27</v>
       </c>
       <c r="B4">
-        <v>0.1020575942901578</v>
+        <v>0.1011781992762632</v>
       </c>
       <c r="C4">
-        <v>0.08785935974388812</v>
+        <v>0.08776298942508712</v>
       </c>
       <c r="D4">
-        <v>0.08759091970802883</v>
+        <v>0.08762134026202249</v>
       </c>
       <c r="E4">
-        <v>0.1017301197815588</v>
+        <v>0.1004907922041731</v>
       </c>
       <c r="F4">
-        <v>0.08189311357013153</v>
+        <v>0.08238622317077363</v>
       </c>
       <c r="G4">
-        <v>0.08896000246192073</v>
+        <v>0.09164525107179181</v>
       </c>
       <c r="H4">
-        <v>0.1805177308707649</v>
+        <v>0.1794567298441801</v>
       </c>
       <c r="I4">
-        <v>0.1522719736514048</v>
+        <v>0.1510013014757943</v>
       </c>
       <c r="J4">
-        <v>0.1424614793486583</v>
+        <v>0.1424198304073822</v>
       </c>
       <c r="K4">
-        <v>0.180359394807826</v>
+        <v>0.175150532538964</v>
       </c>
       <c r="L4">
-        <v>0.1487314679085107</v>
+        <v>0.1475988791882794</v>
       </c>
       <c r="M4">
-        <v>0.1428510392473332</v>
+        <v>0.1427223039092161</v>
       </c>
       <c r="N4">
-        <v>0.1600283688213251</v>
+        <v>0.1554790947547423</v>
       </c>
       <c r="O4">
-        <v>0.1138801724592838</v>
+        <v>0.1079863817025137</v>
       </c>
       <c r="P4">
-        <v>0.07542363225861722</v>
+        <v>0.0786967327387546</v>
       </c>
       <c r="Q4">
-        <v>0.1600283688213251</v>
+        <v>0.1554790947547423</v>
       </c>
       <c r="R4">
-        <v>0.1098547308431051</v>
+        <v>0.1047540835716057</v>
       </c>
       <c r="S4">
-        <v>0.07615299335188513</v>
+        <v>0.07941749656960151</v>
       </c>
       <c r="T4">
-        <v>0.1642009778836675</v>
+        <v>0.1594645402372321</v>
       </c>
       <c r="U4">
-        <v>0.1171815983784434</v>
+        <v>0.1111013229628084</v>
       </c>
       <c r="V4">
-        <v>0.07276340183460943</v>
+        <v>0.06945360897488909</v>
       </c>
       <c r="W4">
-        <v>0.1642009778836675</v>
+        <v>0.1601728829226593</v>
       </c>
       <c r="X4">
-        <v>0.1103770209003428</v>
+        <v>0.1055125191633786</v>
       </c>
       <c r="Y4">
-        <v>0.07366634479915002</v>
+        <v>0.07060066431412124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run scenario and calibration updates
</commit_message>
<xml_diff>
--- a/baseline_hepaus_pars.xlsx
+++ b/baseline_hepaus_pars.xlsx
@@ -540,76 +540,76 @@
         <v>25</v>
       </c>
       <c r="B2">
-        <v>18.48417578649617</v>
+        <v>0.001874215221225689</v>
       </c>
       <c r="C2">
-        <v>336.6093924101857</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>362.6634693098511</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>19.51076314459439</v>
+        <v>0.006498029333137876</v>
       </c>
       <c r="F2">
-        <v>334.373192306528</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>375.4590379768111</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>21.86579141979038</v>
+        <v>0.07201714046726834</v>
       </c>
       <c r="I2">
-        <v>101.9467323267382</v>
+        <v>0.08053147861785559</v>
       </c>
       <c r="J2">
-        <v>709.3782833634586</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>24.87729082341614</v>
+        <v>0.07281075646015447</v>
       </c>
       <c r="L2">
-        <v>104.2095467127555</v>
+        <v>0.06707195875772902</v>
       </c>
       <c r="M2">
-        <v>739.1165571425611</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>1.246137635074309</v>
+        <v>0.01764947577338688</v>
       </c>
       <c r="O2">
-        <v>2.391584698141559</v>
+        <v>0.1057305648110574</v>
       </c>
       <c r="P2">
-        <v>6.982498587646266</v>
+        <v>0.05110793889513847</v>
       </c>
       <c r="Q2">
-        <v>1.246137635074309</v>
+        <v>0.01539884873066284</v>
       </c>
       <c r="R2">
-        <v>2.246608773545434</v>
+        <v>0.1122801476243039</v>
       </c>
       <c r="S2">
-        <v>7.008045735217956</v>
+        <v>0.05191839529364917</v>
       </c>
       <c r="T2">
-        <v>0.6170378583123783</v>
+        <v>0.01449149295716399</v>
       </c>
       <c r="U2">
-        <v>0.6881388067942998</v>
+        <v>0.1057584260281608</v>
       </c>
       <c r="V2">
-        <v>1.068426268265968</v>
+        <v>0.04933866385601611</v>
       </c>
       <c r="W2">
-        <v>0.6167506274594454</v>
+        <v>0.01574999784171747</v>
       </c>
       <c r="X2">
-        <v>0.6210989077072122</v>
+        <v>0.1125046710674354</v>
       </c>
       <c r="Y2">
-        <v>1.02951459833655</v>
+        <v>0.05060047430165641</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -617,76 +617,76 @@
         <v>26</v>
       </c>
       <c r="B3">
-        <v>0.0529089448780045</v>
+        <v>0</v>
       </c>
       <c r="C3">
-        <v>0.01972089867094264</v>
+        <v>0.001046554730485141</v>
       </c>
       <c r="D3">
-        <v>0.01915586180581189</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>0.05109198959676253</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>0.02032383817648103</v>
+        <v>0.003539141918654456</v>
       </c>
       <c r="G3">
-        <v>0.0191811790910337</v>
+        <v>0</v>
       </c>
       <c r="H3">
-        <v>0.05337702947432052</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>0.02204566892543731</v>
+        <v>0.04680863286045586</v>
       </c>
       <c r="J3">
-        <v>0.01888665172255115</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>0.04913473409093153</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>0.02215946038287137</v>
+        <v>0.04001662084563257</v>
       </c>
       <c r="M3">
-        <v>0.01887216237367744</v>
+        <v>0</v>
       </c>
       <c r="N3">
-        <v>0.09804766534194742</v>
+        <v>0</v>
       </c>
       <c r="O3">
-        <v>0.04558949978006736</v>
+        <v>0.07378192745720677</v>
       </c>
       <c r="P3">
-        <v>0.02626313639551821</v>
+        <v>0.02001156611786236</v>
       </c>
       <c r="Q3">
-        <v>0.09804766534194742</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>0.04640989286416679</v>
+        <v>0.0789068659064342</v>
       </c>
       <c r="S3">
-        <v>0.02621573227731289</v>
+        <v>0.02232450547449797</v>
       </c>
       <c r="T3">
-        <v>0.1099217914334042</v>
+        <v>0</v>
       </c>
       <c r="U3">
-        <v>0.05494639158149636</v>
+        <v>0.07191197825374149</v>
       </c>
       <c r="V3">
-        <v>0.02678790885682546</v>
+        <v>0.01715729149576042</v>
       </c>
       <c r="W3">
-        <v>0.1105047786779234</v>
+        <v>0</v>
       </c>
       <c r="X3">
-        <v>0.05626047406919778</v>
+        <v>0.0771100016636177</v>
       </c>
       <c r="Y3">
-        <v>0.02706801197766756</v>
+        <v>0.01848407446277296</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -694,76 +694,76 @@
         <v>27</v>
       </c>
       <c r="B4">
-        <v>0.1011781992762632</v>
+        <v>0</v>
       </c>
       <c r="C4">
-        <v>0.08776298942508712</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>0.08762134026202249</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0.1004907922041731</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>0.08238622317077363</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>0.09164525107179181</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>0.1794567298441801</v>
+        <v>0.02856915313965698</v>
       </c>
       <c r="I4">
-        <v>0.1510013014757943</v>
+        <v>0.03354328833119392</v>
       </c>
       <c r="J4">
-        <v>0.1424198304073822</v>
+        <v>0.0001169917773218092</v>
       </c>
       <c r="K4">
-        <v>0.175150532538964</v>
+        <v>0.02889837061617884</v>
       </c>
       <c r="L4">
-        <v>0.1475988791882794</v>
+        <v>0.02725555195072539</v>
       </c>
       <c r="M4">
-        <v>0.1427223039092161</v>
+        <v>0</v>
       </c>
       <c r="N4">
-        <v>0.1554790947547423</v>
+        <v>0.008829069306242408</v>
       </c>
       <c r="O4">
-        <v>0.1079863817025137</v>
+        <v>0.04909522011805342</v>
       </c>
       <c r="P4">
-        <v>0.0786967327387546</v>
+        <v>0.0183114699703855</v>
       </c>
       <c r="Q4">
-        <v>0.1554790947547423</v>
+        <v>0.008223131141445511</v>
       </c>
       <c r="R4">
-        <v>0.1047540835716057</v>
+        <v>0.05319451351973938</v>
       </c>
       <c r="S4">
-        <v>0.07941749656960151</v>
+        <v>0.01916773438224637</v>
       </c>
       <c r="T4">
-        <v>0.1594645402372321</v>
+        <v>0.007488220337184709</v>
       </c>
       <c r="U4">
-        <v>0.1111013229628084</v>
+        <v>0.04917911062581767</v>
       </c>
       <c r="V4">
-        <v>0.06945360897488909</v>
+        <v>0.01706006061135295</v>
       </c>
       <c r="W4">
-        <v>0.1601728829226593</v>
+        <v>0.007946805154462298</v>
       </c>
       <c r="X4">
-        <v>0.1055125191633786</v>
+        <v>0.05310095774960328</v>
       </c>
       <c r="Y4">
-        <v>0.07060066431412124</v>
+        <v>0.01760178903955496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>